<commit_message>
Daily Satellite Data Update
</commit_message>
<xml_diff>
--- a/Prelety.xlsx
+++ b/Prelety.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="232">
   <si>
     <t>Datum</t>
   </si>
@@ -70,15 +70,6 @@
     <t>Vysoká</t>
   </si>
   <si>
-    <t>20260304--01</t>
-  </si>
-  <si>
-    <t>20260304--02</t>
-  </si>
-  <si>
-    <t>20260304--03</t>
-  </si>
-  <si>
     <t>20260305--01</t>
   </si>
   <si>
@@ -151,513 +142,510 @@
     <t>20260310--04</t>
   </si>
   <si>
-    <t>05:40</t>
-  </si>
-  <si>
-    <t>06:26</t>
-  </si>
-  <si>
-    <t>05:38</t>
-  </si>
-  <si>
-    <t>05:22</t>
+    <t>20260311--01</t>
+  </si>
+  <si>
+    <t>20260311--02</t>
+  </si>
+  <si>
+    <t>20260311--03</t>
+  </si>
+  <si>
+    <t>05:21</t>
   </si>
   <si>
     <t>06:25</t>
   </si>
   <si>
+    <t>05:52</t>
+  </si>
+  <si>
+    <t>04:57</t>
+  </si>
+  <si>
+    <t>06:23</t>
+  </si>
+  <si>
+    <t>06:03</t>
+  </si>
+  <si>
+    <t>02:05</t>
+  </si>
+  <si>
+    <t>04:24</t>
+  </si>
+  <si>
+    <t>06:18</t>
+  </si>
+  <si>
+    <t>06:11</t>
+  </si>
+  <si>
+    <t>03:25</t>
+  </si>
+  <si>
+    <t>03:40</t>
+  </si>
+  <si>
+    <t>06:13</t>
+  </si>
+  <si>
+    <t>06:17</t>
+  </si>
+  <si>
+    <t>04:13</t>
+  </si>
+  <si>
+    <t>02:30</t>
+  </si>
+  <si>
+    <t>06:04</t>
+  </si>
+  <si>
+    <t>06:21</t>
+  </si>
+  <si>
+    <t>04:48</t>
+  </si>
+  <si>
     <t>05:53</t>
   </si>
   <si>
-    <t>04:57</t>
-  </si>
-  <si>
-    <t>06:22</t>
-  </si>
-  <si>
-    <t>06:03</t>
-  </si>
-  <si>
-    <t>02:04</t>
-  </si>
-  <si>
-    <t>04:25</t>
-  </si>
-  <si>
-    <t>06:19</t>
-  </si>
-  <si>
-    <t>06:11</t>
-  </si>
-  <si>
-    <t>03:24</t>
-  </si>
-  <si>
-    <t>03:41</t>
-  </si>
-  <si>
-    <t>06:13</t>
-  </si>
-  <si>
-    <t>06:18</t>
-  </si>
-  <si>
-    <t>04:14</t>
-  </si>
-  <si>
-    <t>02:32</t>
-  </si>
-  <si>
-    <t>06:05</t>
-  </si>
-  <si>
-    <t>06:21</t>
-  </si>
-  <si>
-    <t>04:48</t>
-  </si>
-  <si>
-    <t>05:54</t>
-  </si>
-  <si>
-    <t>06:23</t>
+    <t>06:24</t>
   </si>
   <si>
     <t>05:14</t>
   </si>
   <si>
+    <t>05:39</t>
+  </si>
+  <si>
+    <t>05:35</t>
+  </si>
+  <si>
     <t>00:00</t>
   </si>
   <si>
-    <t>00:59</t>
-  </si>
-  <si>
-    <t>04:31</t>
-  </si>
-  <si>
-    <t>02:55</t>
-  </si>
-  <si>
-    <t>01:12</t>
-  </si>
-  <si>
-    <t>01:43</t>
-  </si>
-  <si>
-    <t>00:11</t>
-  </si>
-  <si>
-    <t>01:14:17</t>
-  </si>
-  <si>
-    <t>02:51:30</t>
-  </si>
-  <si>
-    <t>04:29:10</t>
-  </si>
-  <si>
-    <t>00:35:09</t>
-  </si>
-  <si>
-    <t>02:12:15</t>
-  </si>
-  <si>
-    <t>03:49:52</t>
-  </si>
-  <si>
-    <t>23:55:59</t>
-  </si>
-  <si>
-    <t>01:32:57</t>
-  </si>
-  <si>
-    <t>03:10:31</t>
-  </si>
-  <si>
-    <t>04:48:32</t>
-  </si>
-  <si>
-    <t>23:16:47</t>
-  </si>
-  <si>
-    <t>00:53:36</t>
-  </si>
-  <si>
-    <t>02:31:07</t>
-  </si>
-  <si>
-    <t>04:09:01</t>
-  </si>
-  <si>
-    <t>22:37:33</t>
-  </si>
-  <si>
-    <t>00:14:12</t>
-  </si>
-  <si>
-    <t>01:51:39</t>
-  </si>
-  <si>
-    <t>03:29:28</t>
-  </si>
-  <si>
-    <t>21:58:19</t>
-  </si>
-  <si>
-    <t>23:34:45</t>
-  </si>
-  <si>
-    <t>01:12:08</t>
-  </si>
-  <si>
-    <t>02:49:53</t>
-  </si>
-  <si>
-    <t>22:55:15</t>
-  </si>
-  <si>
-    <t>00:32:33</t>
-  </si>
-  <si>
-    <t>02:10:14</t>
-  </si>
-  <si>
-    <t>22:15:42</t>
-  </si>
-  <si>
-    <t>23:52:54</t>
-  </si>
-  <si>
-    <t>01:16:42</t>
-  </si>
-  <si>
-    <t>02:53:46</t>
-  </si>
-  <si>
-    <t>04:31:36</t>
-  </si>
-  <si>
-    <t>00:37:38</t>
-  </si>
-  <si>
-    <t>02:14:31</t>
-  </si>
-  <si>
-    <t>03:52:15</t>
-  </si>
-  <si>
-    <t>23:58:34</t>
-  </si>
-  <si>
-    <t>01:35:14</t>
-  </si>
-  <si>
-    <t>03:12:52</t>
-  </si>
-  <si>
-    <t>04:52:03</t>
-  </si>
-  <si>
-    <t>23:19:31</t>
-  </si>
-  <si>
-    <t>00:55:53</t>
-  </si>
-  <si>
-    <t>02:33:26</t>
-  </si>
-  <si>
-    <t>04:12:04</t>
-  </si>
-  <si>
-    <t>22:40:30</t>
-  </si>
-  <si>
-    <t>00:16:30</t>
-  </si>
-  <si>
-    <t>01:53:56</t>
-  </si>
-  <si>
-    <t>03:32:16</t>
-  </si>
-  <si>
-    <t>22:01:39</t>
-  </si>
-  <si>
-    <t>23:37:04</t>
-  </si>
-  <si>
-    <t>01:14:24</t>
-  </si>
-  <si>
-    <t>02:52:31</t>
-  </si>
-  <si>
-    <t>22:57:37</t>
-  </si>
-  <si>
-    <t>00:34:49</t>
-  </si>
-  <si>
-    <t>02:12:46</t>
-  </si>
-  <si>
-    <t>22:18:07</t>
-  </si>
-  <si>
-    <t>23:55:10</t>
-  </si>
-  <si>
-    <t>01:19:32</t>
-  </si>
-  <si>
-    <t>02:56:59</t>
-  </si>
-  <si>
-    <t>04:34:25</t>
-  </si>
-  <si>
-    <t>00:40:19</t>
-  </si>
-  <si>
-    <t>02:17:44</t>
-  </si>
-  <si>
-    <t>03:55:11</t>
-  </si>
-  <si>
-    <t>00:01:03</t>
-  </si>
-  <si>
-    <t>01:38:25</t>
-  </si>
-  <si>
-    <t>03:15:53</t>
-  </si>
-  <si>
-    <t>04:53:05</t>
-  </si>
-  <si>
-    <t>23:21:43</t>
-  </si>
-  <si>
-    <t>00:59:02</t>
-  </si>
-  <si>
-    <t>02:36:31</t>
-  </si>
-  <si>
-    <t>04:13:46</t>
-  </si>
-  <si>
-    <t>22:42:20</t>
-  </si>
-  <si>
-    <t>00:19:36</t>
-  </si>
-  <si>
-    <t>01:57:05</t>
-  </si>
-  <si>
-    <t>03:34:23</t>
-  </si>
-  <si>
-    <t>22:02:54</t>
-  </si>
-  <si>
-    <t>23:40:06</t>
-  </si>
-  <si>
-    <t>01:17:35</t>
-  </si>
-  <si>
-    <t>02:54:55</t>
-  </si>
-  <si>
-    <t>23:00:33</t>
-  </si>
-  <si>
-    <t>00:38:01</t>
-  </si>
-  <si>
-    <t>02:15:23</t>
-  </si>
-  <si>
-    <t>22:20:57</t>
-  </si>
-  <si>
-    <t>23:58:22</t>
-  </si>
-  <si>
-    <t>01:22:22</t>
-  </si>
-  <si>
-    <t>03:00:12</t>
-  </si>
-  <si>
-    <t>04:37:14</t>
-  </si>
-  <si>
-    <t>00:43:00</t>
-  </si>
-  <si>
-    <t>02:20:56</t>
-  </si>
-  <si>
-    <t>03:58:08</t>
-  </si>
-  <si>
-    <t>00:03:31</t>
-  </si>
-  <si>
-    <t>01:41:36</t>
-  </si>
-  <si>
-    <t>03:18:55</t>
-  </si>
-  <si>
-    <t>04:54:07</t>
-  </si>
-  <si>
-    <t>23:23:56</t>
-  </si>
-  <si>
-    <t>01:02:12</t>
-  </si>
-  <si>
-    <t>02:39:37</t>
-  </si>
-  <si>
-    <t>04:15:28</t>
-  </si>
-  <si>
-    <t>22:44:11</t>
-  </si>
-  <si>
-    <t>00:22:43</t>
-  </si>
-  <si>
-    <t>02:00:14</t>
-  </si>
-  <si>
-    <t>03:36:30</t>
-  </si>
-  <si>
-    <t>22:04:11</t>
-  </si>
-  <si>
-    <t>23:43:09</t>
-  </si>
-  <si>
-    <t>01:20:45</t>
-  </si>
-  <si>
-    <t>02:57:19</t>
-  </si>
-  <si>
-    <t>23:03:31</t>
-  </si>
-  <si>
-    <t>00:41:12</t>
-  </si>
-  <si>
-    <t>02:18:00</t>
-  </si>
-  <si>
-    <t>22:23:47</t>
-  </si>
-  <si>
-    <t>00:01:35</t>
-  </si>
-  <si>
-    <t>01:24:48</t>
-  </si>
-  <si>
-    <t>03:02:28</t>
-  </si>
-  <si>
-    <t>04:39:40</t>
-  </si>
-  <si>
-    <t>00:45:30</t>
-  </si>
-  <si>
-    <t>02:23:12</t>
-  </si>
-  <si>
-    <t>04:00:30</t>
-  </si>
-  <si>
-    <t>00:06:08</t>
-  </si>
-  <si>
-    <t>01:43:53</t>
-  </si>
-  <si>
-    <t>03:21:15</t>
-  </si>
-  <si>
-    <t>04:57:38</t>
-  </si>
-  <si>
-    <t>23:26:41</t>
-  </si>
-  <si>
-    <t>01:04:29</t>
-  </si>
-  <si>
-    <t>02:41:56</t>
-  </si>
-  <si>
-    <t>04:18:31</t>
-  </si>
-  <si>
-    <t>22:47:09</t>
-  </si>
-  <si>
-    <t>00:25:01</t>
-  </si>
-  <si>
-    <t>02:02:31</t>
-  </si>
-  <si>
-    <t>03:39:17</t>
-  </si>
-  <si>
-    <t>22:07:31</t>
-  </si>
-  <si>
-    <t>23:45:29</t>
-  </si>
-  <si>
-    <t>01:23:02</t>
-  </si>
-  <si>
-    <t>02:59:57</t>
-  </si>
-  <si>
-    <t>23:05:53</t>
-  </si>
-  <si>
-    <t>00:43:28</t>
-  </si>
-  <si>
-    <t>02:20:32</t>
-  </si>
-  <si>
-    <t>22:26:13</t>
-  </si>
-  <si>
-    <t>00:03:50</t>
+    <t>02:54</t>
+  </si>
+  <si>
+    <t>01:11</t>
+  </si>
+  <si>
+    <t>01:44</t>
+  </si>
+  <si>
+    <t>00:10</t>
+  </si>
+  <si>
+    <t>00:35:08</t>
+  </si>
+  <si>
+    <t>02:12:14</t>
+  </si>
+  <si>
+    <t>03:49:51</t>
+  </si>
+  <si>
+    <t>23:55:56</t>
+  </si>
+  <si>
+    <t>01:32:54</t>
+  </si>
+  <si>
+    <t>03:10:28</t>
+  </si>
+  <si>
+    <t>04:48:28</t>
+  </si>
+  <si>
+    <t>23:16:41</t>
+  </si>
+  <si>
+    <t>00:53:30</t>
+  </si>
+  <si>
+    <t>02:31:00</t>
+  </si>
+  <si>
+    <t>04:08:54</t>
+  </si>
+  <si>
+    <t>22:37:24</t>
+  </si>
+  <si>
+    <t>00:14:02</t>
+  </si>
+  <si>
+    <t>01:51:29</t>
+  </si>
+  <si>
+    <t>03:29:18</t>
+  </si>
+  <si>
+    <t>21:58:05</t>
+  </si>
+  <si>
+    <t>23:34:30</t>
+  </si>
+  <si>
+    <t>01:11:53</t>
+  </si>
+  <si>
+    <t>02:49:37</t>
+  </si>
+  <si>
+    <t>22:54:55</t>
+  </si>
+  <si>
+    <t>00:32:12</t>
+  </si>
+  <si>
+    <t>02:09:53</t>
+  </si>
+  <si>
+    <t>22:15:16</t>
+  </si>
+  <si>
+    <t>23:52:27</t>
+  </si>
+  <si>
+    <t>01:30:05</t>
+  </si>
+  <si>
+    <t>21:35:34</t>
+  </si>
+  <si>
+    <t>23:12:38</t>
+  </si>
+  <si>
+    <t>00:37:37</t>
+  </si>
+  <si>
+    <t>02:14:30</t>
+  </si>
+  <si>
+    <t>03:52:14</t>
+  </si>
+  <si>
+    <t>23:58:31</t>
+  </si>
+  <si>
+    <t>01:35:10</t>
+  </si>
+  <si>
+    <t>03:12:48</t>
+  </si>
+  <si>
+    <t>04:51:59</t>
+  </si>
+  <si>
+    <t>23:19:25</t>
+  </si>
+  <si>
+    <t>00:55:47</t>
+  </si>
+  <si>
+    <t>02:33:19</t>
+  </si>
+  <si>
+    <t>04:11:57</t>
+  </si>
+  <si>
+    <t>22:40:21</t>
+  </si>
+  <si>
+    <t>00:16:20</t>
+  </si>
+  <si>
+    <t>01:53:46</t>
+  </si>
+  <si>
+    <t>03:32:06</t>
+  </si>
+  <si>
+    <t>22:01:25</t>
+  </si>
+  <si>
+    <t>23:36:50</t>
+  </si>
+  <si>
+    <t>01:14:09</t>
+  </si>
+  <si>
+    <t>02:52:16</t>
+  </si>
+  <si>
+    <t>22:57:17</t>
+  </si>
+  <si>
+    <t>00:34:28</t>
+  </si>
+  <si>
+    <t>02:12:25</t>
+  </si>
+  <si>
+    <t>22:17:41</t>
+  </si>
+  <si>
+    <t>23:54:43</t>
+  </si>
+  <si>
+    <t>01:32:32</t>
+  </si>
+  <si>
+    <t>21:38:03</t>
+  </si>
+  <si>
+    <t>23:14:54</t>
+  </si>
+  <si>
+    <t>00:40:17</t>
+  </si>
+  <si>
+    <t>02:17:42</t>
+  </si>
+  <si>
+    <t>03:55:10</t>
+  </si>
+  <si>
+    <t>00:00:59</t>
+  </si>
+  <si>
+    <t>01:38:21</t>
+  </si>
+  <si>
+    <t>03:15:50</t>
+  </si>
+  <si>
+    <t>04:53:01</t>
+  </si>
+  <si>
+    <t>23:21:37</t>
+  </si>
+  <si>
+    <t>00:58:56</t>
+  </si>
+  <si>
+    <t>02:36:25</t>
+  </si>
+  <si>
+    <t>04:13:39</t>
+  </si>
+  <si>
+    <t>22:42:11</t>
+  </si>
+  <si>
+    <t>00:19:26</t>
+  </si>
+  <si>
+    <t>01:56:55</t>
+  </si>
+  <si>
+    <t>03:34:12</t>
+  </si>
+  <si>
+    <t>22:02:40</t>
+  </si>
+  <si>
+    <t>23:39:52</t>
+  </si>
+  <si>
+    <t>01:17:20</t>
+  </si>
+  <si>
+    <t>02:54:40</t>
+  </si>
+  <si>
+    <t>23:00:13</t>
+  </si>
+  <si>
+    <t>00:37:40</t>
+  </si>
+  <si>
+    <t>02:15:02</t>
+  </si>
+  <si>
+    <t>22:20:30</t>
+  </si>
+  <si>
+    <t>23:57:55</t>
+  </si>
+  <si>
+    <t>01:35:20</t>
+  </si>
+  <si>
+    <t>21:40:43</t>
+  </si>
+  <si>
+    <t>23:18:06</t>
+  </si>
+  <si>
+    <t>00:42:58</t>
+  </si>
+  <si>
+    <t>02:20:55</t>
+  </si>
+  <si>
+    <t>03:58:06</t>
+  </si>
+  <si>
+    <t>00:03:28</t>
+  </si>
+  <si>
+    <t>01:41:33</t>
+  </si>
+  <si>
+    <t>03:18:51</t>
+  </si>
+  <si>
+    <t>04:54:04</t>
+  </si>
+  <si>
+    <t>23:23:49</t>
+  </si>
+  <si>
+    <t>01:02:05</t>
+  </si>
+  <si>
+    <t>02:39:30</t>
+  </si>
+  <si>
+    <t>04:15:22</t>
+  </si>
+  <si>
+    <t>22:44:01</t>
+  </si>
+  <si>
+    <t>00:22:33</t>
+  </si>
+  <si>
+    <t>02:00:03</t>
+  </si>
+  <si>
+    <t>03:36:19</t>
+  </si>
+  <si>
+    <t>22:03:55</t>
+  </si>
+  <si>
+    <t>23:42:54</t>
+  </si>
+  <si>
+    <t>01:20:30</t>
+  </si>
+  <si>
+    <t>02:57:04</t>
+  </si>
+  <si>
+    <t>23:03:10</t>
+  </si>
+  <si>
+    <t>00:40:52</t>
+  </si>
+  <si>
+    <t>02:17:39</t>
+  </si>
+  <si>
+    <t>22:23:20</t>
+  </si>
+  <si>
+    <t>00:01:07</t>
+  </si>
+  <si>
+    <t>01:38:07</t>
+  </si>
+  <si>
+    <t>21:43:24</t>
+  </si>
+  <si>
+    <t>23:21:18</t>
+  </si>
+  <si>
+    <t>00:45:28</t>
+  </si>
+  <si>
+    <t>02:23:11</t>
+  </si>
+  <si>
+    <t>04:00:29</t>
+  </si>
+  <si>
+    <t>00:06:04</t>
+  </si>
+  <si>
+    <t>01:43:49</t>
+  </si>
+  <si>
+    <t>03:21:12</t>
+  </si>
+  <si>
+    <t>04:57:35</t>
+  </si>
+  <si>
+    <t>23:26:34</t>
+  </si>
+  <si>
+    <t>01:04:23</t>
+  </si>
+  <si>
+    <t>02:41:49</t>
+  </si>
+  <si>
+    <t>04:18:24</t>
+  </si>
+  <si>
+    <t>22:46:59</t>
+  </si>
+  <si>
+    <t>00:24:51</t>
+  </si>
+  <si>
+    <t>02:02:20</t>
+  </si>
+  <si>
+    <t>03:39:07</t>
+  </si>
+  <si>
+    <t>22:07:17</t>
+  </si>
+  <si>
+    <t>23:45:14</t>
+  </si>
+  <si>
+    <t>01:22:47</t>
+  </si>
+  <si>
+    <t>02:59:42</t>
+  </si>
+  <si>
+    <t>23:05:33</t>
+  </si>
+  <si>
+    <t>00:43:07</t>
+  </si>
+  <si>
+    <t>02:20:11</t>
+  </si>
+  <si>
+    <t>22:25:46</t>
+  </si>
+  <si>
+    <t>00:03:23</t>
+  </si>
+  <si>
+    <t>01:40:33</t>
+  </si>
+  <si>
+    <t>21:45:54</t>
+  </si>
+  <si>
+    <t>23:23:34</t>
   </si>
   <si>
     <t>0°</t>
   </si>
   <si>
-    <t>16°</t>
-  </si>
-  <si>
     <t>6°</t>
   </si>
   <si>
@@ -682,34 +670,28 @@
     <t>3°</t>
   </si>
   <si>
-    <t>02:59:13</t>
-  </si>
-  <si>
-    <t>04:32:43</t>
-  </si>
-  <si>
-    <t>02:21:43</t>
-  </si>
-  <si>
-    <t>03:55:13</t>
-  </si>
-  <si>
-    <t>03:17:43</t>
-  </si>
-  <si>
-    <t>04:51:13</t>
-  </si>
-  <si>
-    <t>02:40:15</t>
-  </si>
-  <si>
-    <t>04:13:45</t>
-  </si>
-  <si>
-    <t>03:36:19</t>
-  </si>
-  <si>
-    <t>02:58:57</t>
+    <t>02:21:42</t>
+  </si>
+  <si>
+    <t>03:55:12</t>
+  </si>
+  <si>
+    <t>03:17:40</t>
+  </si>
+  <si>
+    <t>04:51:09</t>
+  </si>
+  <si>
+    <t>02:40:08</t>
+  </si>
+  <si>
+    <t>04:13:38</t>
+  </si>
+  <si>
+    <t>03:36:09</t>
+  </si>
+  <si>
+    <t>02:58:42</t>
   </si>
   <si>
     <t>B</t>
@@ -761,7 +743,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -776,13 +758,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF0707F"/>
+        <fgColor rgb="FFF0B070"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDDE8F4"/>
+        <fgColor rgb="FFAAC5E3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -800,7 +782,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFCCDCEE"/>
+        <fgColor rgb="FF6AD26A"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -812,13 +794,67 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF88AED8"/>
+        <fgColor rgb="FFF0707F"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6AD26A"/>
+        <fgColor rgb="FF99BADE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCDCEE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F9FC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6EEF7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD4E2F1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF80A9D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF77A3D3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6697CD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDE8F4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -830,31 +866,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF0B070"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF6697CD"/>
+        <fgColor rgb="FFC4D7EC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFB2CBE6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFBBD1E9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF77A3D3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -895,7 +913,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -952,6 +970,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1433,55 +1469,55 @@
         <v>18</v>
       </c>
       <c r="B2" s="2">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="L2" s="4">
-        <v>-39</v>
+        <v>-42.1</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="O2" s="6">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="P2" s="7">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="Q2" s="8">
         <v>0</v>
       </c>
-      <c r="R2" s="9">
-        <v>44</v>
+      <c r="R2" s="8">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -1489,55 +1525,55 @@
         <v>19</v>
       </c>
       <c r="B3" s="2">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>46</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="L3" s="4">
-        <v>-26.5</v>
+        <v>-31.6</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="O3" s="6">
-        <v>51</v>
-      </c>
-      <c r="P3" s="7">
-        <v>80</v>
+        <v>21</v>
+      </c>
+      <c r="P3" s="9">
+        <v>45</v>
       </c>
       <c r="Q3" s="8">
         <v>0</v>
       </c>
-      <c r="R3" s="10">
-        <v>68</v>
+      <c r="R3" s="8">
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -1545,55 +1581,55 @@
         <v>20</v>
       </c>
       <c r="B4" s="2">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>47</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="L4" s="4">
-        <v>-11.7</v>
+        <v>-17.5</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="O4" s="6">
-        <v>84</v>
-      </c>
-      <c r="P4" s="7">
-        <v>80</v>
-      </c>
-      <c r="Q4" s="11">
-        <v>13</v>
-      </c>
-      <c r="R4" s="12">
-        <v>30</v>
+        <v>230</v>
+      </c>
+      <c r="O4" s="10">
+        <v>2</v>
+      </c>
+      <c r="P4" s="9">
+        <v>45</v>
+      </c>
+      <c r="Q4" s="8">
+        <v>0</v>
+      </c>
+      <c r="R4" s="8">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -1601,49 +1637,49 @@
         <v>21</v>
       </c>
       <c r="B5" s="2">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>48</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="L5" s="4">
-        <v>-42.1</v>
+        <v>-44.1</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O5" s="13">
-        <v>7</v>
-      </c>
-      <c r="P5" s="14">
-        <v>7</v>
+        <v>229</v>
+      </c>
+      <c r="O5" s="10">
+        <v>0</v>
+      </c>
+      <c r="P5" s="8">
+        <v>0</v>
       </c>
       <c r="Q5" s="8">
         <v>0</v>
@@ -1663,39 +1699,39 @@
         <v>49</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>224</v>
+        <v>78</v>
       </c>
       <c r="L6" s="4">
-        <v>-31.6</v>
+        <v>-36.2</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O6" s="13">
+        <v>229</v>
+      </c>
+      <c r="O6" s="10">
         <v>0</v>
       </c>
       <c r="P6" s="8">
@@ -1713,45 +1749,45 @@
         <v>23</v>
       </c>
       <c r="B7" s="2">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>50</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="L7" s="4">
-        <v>-17.5</v>
+        <v>-23.1</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="O7" s="13">
+        <v>230</v>
+      </c>
+      <c r="O7" s="10">
         <v>0</v>
       </c>
       <c r="P7" s="8">
@@ -1769,45 +1805,45 @@
         <v>24</v>
       </c>
       <c r="B8" s="2">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>83</v>
+        <v>221</v>
       </c>
       <c r="L8" s="4">
-        <v>-44.1</v>
+        <v>-8</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O8" s="13">
+        <v>231</v>
+      </c>
+      <c r="O8" s="10">
         <v>0</v>
       </c>
       <c r="P8" s="8">
@@ -1825,46 +1861,46 @@
         <v>25</v>
       </c>
       <c r="B9" s="2">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>52</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="L9" s="4">
-        <v>-36.2</v>
+        <v>-44.7</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O9" s="13">
-        <v>0</v>
+        <v>229</v>
+      </c>
+      <c r="O9" s="10">
+        <v>2</v>
       </c>
       <c r="P9" s="8">
         <v>0</v>
@@ -1873,7 +1909,7 @@
         <v>0</v>
       </c>
       <c r="R9" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -1881,46 +1917,46 @@
         <v>26</v>
       </c>
       <c r="B10" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="K10" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="L10" s="4">
+        <v>-39.8</v>
+      </c>
+      <c r="M10" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="L10" s="4">
-        <v>-23.1</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>233</v>
-      </c>
       <c r="N10" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="O10" s="13">
-        <v>0</v>
+        <v>229</v>
+      </c>
+      <c r="O10" s="10">
+        <v>2</v>
       </c>
       <c r="P10" s="8">
         <v>0</v>
@@ -1929,7 +1965,7 @@
         <v>0</v>
       </c>
       <c r="R10" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -1937,46 +1973,46 @@
         <v>27</v>
       </c>
       <c r="B11" s="2">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="L11" s="4">
-        <v>-8</v>
+        <v>-28.3</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="O11" s="13">
-        <v>0</v>
+        <v>229</v>
+      </c>
+      <c r="O11" s="10">
+        <v>2</v>
       </c>
       <c r="P11" s="8">
         <v>0</v>
@@ -1985,7 +2021,7 @@
         <v>0</v>
       </c>
       <c r="R11" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:18">
@@ -1993,46 +2029,46 @@
         <v>28</v>
       </c>
       <c r="B12" s="2">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>55</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>87</v>
+        <v>223</v>
       </c>
       <c r="L12" s="4">
-        <v>-44.7</v>
+        <v>-13.9</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O12" s="13">
-        <v>3</v>
+        <v>231</v>
+      </c>
+      <c r="O12" s="10">
+        <v>16</v>
       </c>
       <c r="P12" s="8">
         <v>0</v>
@@ -2040,8 +2076,8 @@
       <c r="Q12" s="8">
         <v>0</v>
       </c>
-      <c r="R12" s="8">
-        <v>2</v>
+      <c r="R12" s="11">
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -2049,55 +2085,55 @@
         <v>29</v>
       </c>
       <c r="B13" s="2">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L13" s="4">
-        <v>-39.8</v>
+        <v>-43.8</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O13" s="15">
-        <v>22</v>
+        <v>231</v>
+      </c>
+      <c r="O13" s="12">
+        <v>75</v>
       </c>
       <c r="P13" s="8">
         <v>0</v>
       </c>
-      <c r="Q13" s="8">
-        <v>0</v>
-      </c>
-      <c r="R13" s="16">
-        <v>11</v>
+      <c r="Q13" s="13">
+        <v>40</v>
+      </c>
+      <c r="R13" s="14">
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:18">
@@ -2105,55 +2141,55 @@
         <v>30</v>
       </c>
       <c r="B14" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>57</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>228</v>
+        <v>86</v>
       </c>
       <c r="L14" s="4">
-        <v>-28.3</v>
+        <v>-42.4</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O14" s="15">
-        <v>25</v>
+        <v>229</v>
+      </c>
+      <c r="O14" s="12">
+        <v>95</v>
       </c>
       <c r="P14" s="8">
         <v>0</v>
       </c>
-      <c r="Q14" s="8">
-        <v>0</v>
-      </c>
-      <c r="R14" s="14">
-        <v>3</v>
+      <c r="Q14" s="9">
+        <v>43</v>
+      </c>
+      <c r="R14" s="15">
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -2161,55 +2197,55 @@
         <v>31</v>
       </c>
       <c r="B15" s="2">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>58</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="K15" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="L15" s="4">
+        <v>-33.2</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="N15" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="L15" s="4">
-        <v>-13.9</v>
-      </c>
-      <c r="M15" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="N15" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="O15" s="13">
-        <v>4</v>
+      <c r="O15" s="12">
+        <v>100</v>
       </c>
       <c r="P15" s="8">
         <v>0</v>
       </c>
-      <c r="Q15" s="8">
-        <v>0</v>
-      </c>
-      <c r="R15" s="8">
-        <v>0</v>
+      <c r="Q15" s="16">
+        <v>86</v>
+      </c>
+      <c r="R15" s="17">
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:18">
@@ -2217,55 +2253,55 @@
         <v>32</v>
       </c>
       <c r="B16" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>59</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>91</v>
+        <v>224</v>
       </c>
       <c r="L16" s="4">
-        <v>-43.8</v>
+        <v>-19.6</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="O16" s="15">
-        <v>39</v>
+        <v>230</v>
+      </c>
+      <c r="O16" s="12">
+        <v>100</v>
       </c>
       <c r="P16" s="8">
         <v>0</v>
       </c>
-      <c r="Q16" s="14">
-        <v>5</v>
-      </c>
-      <c r="R16" s="8">
-        <v>0</v>
+      <c r="Q16" s="18">
+        <v>75</v>
+      </c>
+      <c r="R16" s="17">
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:18">
@@ -2273,52 +2309,52 @@
         <v>33</v>
       </c>
       <c r="B17" s="2">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>60</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="L17" s="4">
-        <v>-42.4</v>
+        <v>-41.5</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O17" s="13">
-        <v>17</v>
+        <v>231</v>
+      </c>
+      <c r="O17" s="6">
+        <v>25</v>
       </c>
       <c r="P17" s="8">
         <v>0</v>
       </c>
-      <c r="Q17" s="14">
-        <v>3</v>
+      <c r="Q17" s="19">
+        <v>25</v>
       </c>
       <c r="R17" s="8">
         <v>0</v>
@@ -2329,52 +2365,52 @@
         <v>34</v>
       </c>
       <c r="B18" s="2">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>61</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="L18" s="4">
-        <v>-33.2</v>
+        <v>-43.7</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O18" s="13">
-        <v>16</v>
+        <v>229</v>
+      </c>
+      <c r="O18" s="6">
+        <v>28</v>
       </c>
       <c r="P18" s="8">
         <v>0</v>
       </c>
-      <c r="Q18" s="16">
-        <v>12</v>
+      <c r="Q18" s="19">
+        <v>27</v>
       </c>
       <c r="R18" s="8">
         <v>0</v>
@@ -2385,52 +2421,52 @@
         <v>35</v>
       </c>
       <c r="B19" s="2">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>62</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>230</v>
+        <v>91</v>
       </c>
       <c r="L19" s="4">
-        <v>-19.6</v>
+        <v>-37.3</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="O19" s="15">
-        <v>29</v>
+        <v>229</v>
+      </c>
+      <c r="O19" s="6">
+        <v>25</v>
       </c>
       <c r="P19" s="8">
         <v>0</v>
       </c>
-      <c r="Q19" s="12">
-        <v>29</v>
+      <c r="Q19" s="20">
+        <v>20</v>
       </c>
       <c r="R19" s="8">
         <v>0</v>
@@ -2441,52 +2477,52 @@
         <v>36</v>
       </c>
       <c r="B20" s="2">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>63</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>95</v>
+        <v>225</v>
       </c>
       <c r="L20" s="4">
-        <v>-41.5</v>
+        <v>-25.1</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="O20" s="6">
-        <v>75</v>
-      </c>
-      <c r="P20" s="17">
-        <v>55</v>
-      </c>
-      <c r="Q20" s="8">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="P20" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="21">
+        <v>10</v>
       </c>
       <c r="R20" s="8">
         <v>0</v>
@@ -2497,55 +2533,55 @@
         <v>37</v>
       </c>
       <c r="B21" s="2">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>64</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="L21" s="4">
+        <v>-43.5</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="O21" s="12">
+        <v>90</v>
+      </c>
+      <c r="P21" s="14">
         <v>70</v>
       </c>
-      <c r="E21" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="L21" s="4">
-        <v>-43.6</v>
-      </c>
-      <c r="M21" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O21" s="6">
-        <v>80</v>
-      </c>
-      <c r="P21" s="17">
-        <v>55</v>
-      </c>
       <c r="Q21" s="8">
         <v>0</v>
       </c>
       <c r="R21" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:18">
@@ -2553,55 +2589,55 @@
         <v>38</v>
       </c>
       <c r="B22" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>65</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L22" s="4">
-        <v>-37.3</v>
+        <v>-40.4</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O22" s="6">
+        <v>229</v>
+      </c>
+      <c r="O22" s="12">
+        <v>96</v>
+      </c>
+      <c r="P22" s="22">
         <v>79</v>
       </c>
-      <c r="P22" s="18">
-        <v>59</v>
-      </c>
-      <c r="Q22" s="8">
-        <v>0</v>
+      <c r="Q22" s="23">
+        <v>3</v>
       </c>
       <c r="R22" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:18">
@@ -2609,55 +2645,55 @@
         <v>39</v>
       </c>
       <c r="B23" s="2">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>66</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>231</v>
+        <v>95</v>
       </c>
       <c r="L23" s="4">
-        <v>-25</v>
+        <v>-30.2</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O23" s="6">
+        <v>229</v>
+      </c>
+      <c r="O23" s="12">
+        <v>82</v>
+      </c>
+      <c r="P23" s="18">
         <v>74</v>
       </c>
-      <c r="P23" s="18">
-        <v>59</v>
-      </c>
       <c r="Q23" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R23" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:18">
@@ -2665,55 +2701,55 @@
         <v>40</v>
       </c>
       <c r="B24" s="2">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>67</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="L24" s="4">
-        <v>-43.5</v>
+        <v>-41.8</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O24" s="15">
-        <v>39</v>
-      </c>
-      <c r="P24" s="14">
-        <v>3</v>
-      </c>
-      <c r="Q24" s="19">
-        <v>20</v>
-      </c>
-      <c r="R24" s="11">
-        <v>13</v>
+        <v>229</v>
+      </c>
+      <c r="O24" s="10">
+        <v>4</v>
+      </c>
+      <c r="P24" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="8">
+        <v>0</v>
+      </c>
+      <c r="R24" s="8">
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:18">
@@ -2721,55 +2757,55 @@
         <v>41</v>
       </c>
       <c r="B25" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="L25" s="4">
-        <v>-40.4</v>
+        <v>-42.3</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O25" s="15">
-        <v>34</v>
+        <v>229</v>
+      </c>
+      <c r="O25" s="10">
+        <v>4</v>
       </c>
       <c r="P25" s="8">
         <v>0</v>
       </c>
-      <c r="Q25" s="16">
-        <v>11</v>
-      </c>
-      <c r="R25" s="19">
-        <v>21</v>
+      <c r="Q25" s="8">
+        <v>0</v>
+      </c>
+      <c r="R25" s="8">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:18">
@@ -2777,55 +2813,55 @@
         <v>42</v>
       </c>
       <c r="B26" s="2">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C26" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="E26" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="I26" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="J26" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="J26" s="3" t="s">
-        <v>212</v>
-      </c>
       <c r="K26" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="L26" s="4">
-        <v>-30.2</v>
+        <v>-34.6</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O26" s="6">
-        <v>52</v>
-      </c>
-      <c r="P26" s="14">
+        <v>229</v>
+      </c>
+      <c r="O26" s="10">
         <v>4</v>
       </c>
-      <c r="Q26" s="19">
-        <v>22</v>
-      </c>
-      <c r="R26" s="11">
-        <v>17</v>
+      <c r="P26" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="8">
+        <v>0</v>
+      </c>
+      <c r="R26" s="8">
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:18">
@@ -2833,55 +2869,55 @@
         <v>43</v>
       </c>
       <c r="B27" s="2">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>45</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L27" s="4">
-        <v>-41.8</v>
+        <v>-38.8</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O27" s="15">
-        <v>20</v>
-      </c>
-      <c r="P27" s="14">
-        <v>5</v>
-      </c>
-      <c r="Q27" s="19">
-        <v>20</v>
-      </c>
-      <c r="R27" s="11">
-        <v>16</v>
+        <v>229</v>
+      </c>
+      <c r="O27" s="12">
+        <v>82</v>
+      </c>
+      <c r="P27" s="7">
+        <v>49</v>
+      </c>
+      <c r="Q27" s="24">
+        <v>65</v>
+      </c>
+      <c r="R27" s="22">
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:18">
@@ -2889,55 +2925,55 @@
         <v>44</v>
       </c>
       <c r="B28" s="2">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="L28" s="4">
-        <v>-42.3</v>
+        <v>-42.8</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="O28" s="13">
-        <v>10</v>
-      </c>
-      <c r="P28" s="14">
-        <v>3</v>
-      </c>
-      <c r="Q28" s="16">
-        <v>10</v>
-      </c>
-      <c r="R28" s="16">
-        <v>10</v>
+        <v>229</v>
+      </c>
+      <c r="O28" s="12">
+        <v>91</v>
+      </c>
+      <c r="P28" s="25">
+        <v>56</v>
+      </c>
+      <c r="Q28" s="24">
+        <v>65</v>
+      </c>
+      <c r="R28" s="18">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>